<commit_message>
chore: remove temporary Excel file and update main fixture schedule; ensure only the latest version is retained for clarity and consistency
</commit_message>
<xml_diff>
--- a/LA_Badminton_Club_Final_Fixture_Schedule.xlsx
+++ b/LA_Badminton_Club_Final_Fixture_Schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\skyga\OneDrive\Documents\Personal Projects\TournamnetWeb\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7A64064-439B-4640-8478-A37F0B61EA04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{524710FC-687A-4820-8C8B-5F2FF941BE5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="129">
   <si>
     <t>Time</t>
   </si>
@@ -350,9 +350,6 @@
     <t>Velmurugan / Gokul</t>
   </si>
   <si>
-    <t>Niranjan / Sky</t>
-  </si>
-  <si>
     <t>4</t>
   </si>
   <si>
@@ -398,9 +395,6 @@
     <t>Rajeshwar</t>
   </si>
   <si>
-    <t>sky</t>
-  </si>
-  <si>
     <t>Tharun / Surya</t>
   </si>
   <si>
@@ -411,6 +405,12 @@
   </si>
   <si>
     <t>Eshanth / S Asfer</t>
+  </si>
+  <si>
+    <t>Samyukth Sakthivel</t>
+  </si>
+  <si>
+    <t>Niranjan / Samyukth Sakthivel</t>
   </si>
 </sst>
 </file>
@@ -1171,7 +1171,7 @@
         <v>85</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -1270,7 +1270,7 @@
         <v>96</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
@@ -1303,7 +1303,7 @@
         <v>103</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
@@ -1325,7 +1325,7 @@
         <v>103</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
@@ -1358,7 +1358,7 @@
         <v>105</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>108</v>
+        <v>128</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
@@ -1366,10 +1366,10 @@
         <v>99</v>
       </c>
       <c r="B22" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>109</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
@@ -1377,10 +1377,10 @@
         <v>99</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
@@ -1388,109 +1388,109 @@
         <v>99</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B25" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="C25" s="2" t="s">
         <v>114</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B26" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="B26" s="2" t="s">
-        <v>114</v>
-      </c>
       <c r="C26" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B27" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="B27" s="2" t="s">
-        <v>114</v>
-      </c>
       <c r="C27" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="B28" s="2" t="s">
-        <v>114</v>
-      </c>
       <c r="C28" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B29" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C29" s="2" t="s">
         <v>119</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="B33" s="5" t="s">
-        <v>114</v>
+        <v>99</v>
+      </c>
+      <c r="B33" s="5">
+        <v>1</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>